<commit_message>
calibrate: align year-end roster and events to implemented-state rule (三源校准)
- 呼伦贝尔 PL-2001-006: approved 2001-10-10 (国函〔2001〕130号), implemented
  2002-02 -> 2001 year-end 呼伦贝尔盟, 2002 onward 呼伦贝尔市
- 中卫 PL-2003-006: approved 2003-12-31 (国函〔2003〕139号), implemented
  2004-02-06 (宁政发〔2004〕12号) -> 2003 not_established, 2004 onward active
- Backfill doc numbers: 定西 国函〔2003〕46号, 吕梁 国函〔2003〕112号
- Add missing county event 海拉尔市->海拉尔区 (WIKI-COUNTY-2001-01-036)
- Master xlsx, timing/entity-year-end overrides updated; full build chain,
  release artifacts, docs site data and SHA256SUMS regenerated
</commit_message>
<xml_diff>
--- a/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
+++ b/data/releases/v4.0/china_city_entity_master_V4.0.xlsx
@@ -2769,7 +2769,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>1987-2000 呼伦贝尔盟; 2001-2026 呼伦贝尔市</t>
+          <t>1987-2001 呼伦贝尔盟; 2002-2026 呼伦贝尔市</t>
         </is>
       </c>
       <c r="O32" t="n">
@@ -24196,7 +24196,7 @@
         </is>
       </c>
       <c r="H326" t="n">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="I326" t="n">
         <v>2026</v>
@@ -24223,7 +24223,7 @@
       </c>
       <c r="N326" t="inlineStr">
         <is>
-          <t>1987-2002 [not_established]; 2003-2026 中卫市</t>
+          <t>1987-2003 [not_established]; 2004-2026 中卫市</t>
         </is>
       </c>
       <c r="O326" t="n">

</xml_diff>